<commit_message>
Add SOH report for 2026-10-30
</commit_message>
<xml_diff>
--- a/reports/SOH_30_10_2026.xlsx
+++ b/reports/SOH_30_10_2026.xlsx
@@ -1453,7 +1453,7 @@
         <v>816</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>1</v>
+        <v>10850</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         <v>888</v>
       </c>
       <c r="E232" s="3" t="n">
-        <v>1</v>
+        <v>9450</v>
       </c>
       <c r="F232" t="inlineStr">
         <is>
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="D267" s="2" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E267" s="3" t="n">
         <v>1</v>
@@ -8538,7 +8538,7 @@
         </is>
       </c>
       <c r="D292" s="2" t="n">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E292" s="3" t="n">
         <v>1</v>
@@ -8766,7 +8766,7 @@
         </is>
       </c>
       <c r="D301" s="2" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E301" s="3" t="n">
         <v>1</v>
@@ -8822,7 +8822,7 @@
         </is>
       </c>
       <c r="D303" s="2" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E303" s="3" t="n">
         <v>1</v>
@@ -9074,7 +9074,7 @@
         </is>
       </c>
       <c r="D312" s="2" t="n">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E312" s="3" t="n">
         <v>1</v>
@@ -9410,7 +9410,7 @@
         </is>
       </c>
       <c r="D324" s="2" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E324" s="3" t="n">
         <v>1</v>
@@ -10082,7 +10082,7 @@
         </is>
       </c>
       <c r="D348" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E348" s="3" t="n">
         <v>4000</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="D355" s="2" t="n">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E355" s="3" t="n">
         <v>3000</v>
@@ -10306,7 +10306,7 @@
         </is>
       </c>
       <c r="D356" s="2" t="n">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="E356" s="3" t="n">
         <v>3000</v>
@@ -10558,7 +10558,7 @@
         </is>
       </c>
       <c r="D365" s="2" t="n">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="E365" s="3" t="n">
         <v>12500</v>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="D373" s="2" t="n">
-        <v>859</v>
+        <v>841</v>
       </c>
       <c r="E373" s="3" t="n">
         <v>40000</v>
@@ -10810,7 +10810,7 @@
         </is>
       </c>
       <c r="D374" s="2" t="n">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="E374" s="3" t="n">
         <v>10500</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="D375" s="2" t="n">
-        <v>594</v>
+        <v>576</v>
       </c>
       <c r="E375" s="3" t="n">
         <v>40000</v>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D377" s="2" t="n">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="E377" s="3" t="n">
         <v>40000</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="D379" s="2" t="n">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E379" s="3" t="n">
         <v>40000</v>
@@ -11370,7 +11370,7 @@
         </is>
       </c>
       <c r="D394" s="2" t="n">
-        <v>-9</v>
+        <v>-1</v>
       </c>
       <c r="E394" s="3" t="n">
         <v>26500</v>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="D399" s="2" t="n">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E399" s="3" t="n">
         <v>51000</v>
@@ -11566,7 +11566,7 @@
         </is>
       </c>
       <c r="D401" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E401" s="3" t="n">
         <v>5000</v>
@@ -11930,7 +11930,7 @@
         </is>
       </c>
       <c r="D414" s="2" t="n">
-        <v>2417</v>
+        <v>2416</v>
       </c>
       <c r="E414" s="3" t="n">
         <v>3876</v>
@@ -12154,7 +12154,7 @@
         </is>
       </c>
       <c r="D422" s="2" t="n">
-        <v>-50</v>
+        <v>-56</v>
       </c>
       <c r="E422" s="3" t="n">
         <v>8000</v>
@@ -12378,7 +12378,7 @@
         </is>
       </c>
       <c r="D430" s="2" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E430" s="3" t="n">
         <v>6750</v>
@@ -13022,7 +13022,7 @@
         </is>
       </c>
       <c r="D453" s="2" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="E453" s="3" t="n">
         <v>36000</v>
@@ -13501,7 +13501,7 @@
         <v>48</v>
       </c>
       <c r="E470" s="3" t="n">
-        <v>1</v>
+        <v>32200</v>
       </c>
       <c r="F470" t="inlineStr">
         <is>
@@ -18846,7 +18846,7 @@
         </is>
       </c>
       <c r="D661" s="2" t="n">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="E661" s="3" t="n">
         <v>25000</v>
@@ -18874,7 +18874,7 @@
         </is>
       </c>
       <c r="D662" s="2" t="n">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E662" s="3" t="n">
         <v>1</v>
@@ -20386,7 +20386,7 @@
         </is>
       </c>
       <c r="D716" s="2" t="n">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="E716" s="3" t="n">
         <v>21000</v>
@@ -20890,7 +20890,7 @@
         </is>
       </c>
       <c r="D734" s="2" t="n">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="E734" s="3" t="n">
         <v>6968</v>
@@ -21226,7 +21226,7 @@
         </is>
       </c>
       <c r="D746" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E746" s="3" t="n">
         <v>7521</v>
@@ -25006,7 +25006,7 @@
         </is>
       </c>
       <c r="D881" s="2" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E881" s="3" t="n">
         <v>25015</v>
@@ -25594,7 +25594,7 @@
         </is>
       </c>
       <c r="D902" s="2" t="n">
-        <v>586</v>
+        <v>572</v>
       </c>
       <c r="E902" s="3" t="n">
         <v>26000</v>
@@ -25650,7 +25650,7 @@
         </is>
       </c>
       <c r="D904" s="2" t="n">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E904" s="3" t="n">
         <v>1</v>
@@ -25958,7 +25958,7 @@
         </is>
       </c>
       <c r="D915" s="2" t="n">
-        <v>718</v>
+        <v>670</v>
       </c>
       <c r="E915" s="3" t="n">
         <v>12500</v>
@@ -26154,7 +26154,7 @@
         </is>
       </c>
       <c r="D922" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E922" s="3" t="n">
         <v>18059</v>
@@ -26210,7 +26210,7 @@
         </is>
       </c>
       <c r="D924" s="2" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E924" s="3" t="n">
         <v>21000</v>
@@ -26238,7 +26238,7 @@
         </is>
       </c>
       <c r="D925" s="2" t="n">
-        <v>1339</v>
+        <v>1331</v>
       </c>
       <c r="E925" s="3" t="n">
         <v>1195</v>
@@ -30214,7 +30214,7 @@
         </is>
       </c>
       <c r="D1067" s="2" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="E1067" s="3" t="n">
         <v>52044</v>
@@ -37383,7 +37383,7 @@
         </is>
       </c>
       <c r="D1323" s="2" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E1323" s="3" t="n">
         <v>16220</v>

</xml_diff>